<commit_message>
Refine three-way presentation workbook layout
</commit_message>
<xml_diff>
--- a/doc/presentation-data/gpg_deferred_adaptive_rtx5090_k1m.xlsx
+++ b/doc/presentation-data/gpg_deferred_adaptive_rtx5090_k1m.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Methodology" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Three-way comparison'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Three-way comparison'!$A$1:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
-    <numFmt numFmtId="165" formatCode="0.000x"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -83,8 +82,8 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -163,15 +162,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GPGDeferredAdaptive" displayName="GPGDeferredAdaptive" ref="A1:F11" headerRowCount="1">
-  <autoFilter ref="A1:F11"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GPGDeferredAdaptive" displayName="GPGDeferredAdaptive" ref="A1:D11" headerRowCount="1">
+  <autoFilter ref="A1:D11"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="Benchmark"/>
     <tableColumn id="2" name="GPG (ms)"/>
-    <tableColumn id="3" name="Deferred (ms)"/>
-    <tableColumn id="4" name="Deferred speedup"/>
-    <tableColumn id="5" name="Adaptive defer (ms)"/>
-    <tableColumn id="6" name="Adaptive speedup"/>
+    <tableColumn id="3" name="Deferred: ms (speedup)"/>
+    <tableColumn id="4" name="Adaptive defer: ms (speedup)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -466,15 +463,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -490,22 +485,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Deferred (ms)</t>
+          <t>Deferred: ms (speedup)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Deferred speedup</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Adaptive defer (ms)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Adaptive speedup</t>
+          <t>Adaptive defer: ms (speedup)</t>
         </is>
       </c>
     </row>
@@ -518,17 +503,15 @@
       <c r="B2" s="3" t="n">
         <v>372.665</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>116.226</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>3.206382</v>
-      </c>
-      <c r="E2" s="3" t="n">
-        <v>115.575</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>3.224443</v>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>116.226 (3.206x)</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>115.575 (3.224x)</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -540,17 +523,15 @@
       <c r="B3" s="3" t="n">
         <v>259.342</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>106.488</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>2.435411</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>64.09327</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>4.046322</v>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>106.488 (2.435x)</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>64.093 (4.046x)</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -562,17 +543,15 @@
       <c r="B4" s="3" t="n">
         <v>4795.25</v>
       </c>
-      <c r="C4" s="3" t="n">
-        <v>1991.45</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>2.407919</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>888.7236799999999</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>5.395659</v>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1,991.450 (2.408x)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>888.724 (5.396x)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -584,17 +563,15 @@
       <c r="B5" s="3" t="n">
         <v>151.353</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>78.4636</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>1.928958</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>84.7291</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>1.786317</v>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>78.464 (1.929x)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>84.729 (1.786x)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -606,17 +583,15 @@
       <c r="B6" s="3" t="n">
         <v>157.362</v>
       </c>
-      <c r="C6" s="3" t="n">
-        <v>110.409</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>1.425264</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>109.0203</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>1.443419</v>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>110.409 (1.425x)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>109.020 (1.443x)</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -628,17 +603,15 @@
       <c r="B7" s="3" t="n">
         <v>7.2124</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>24.307</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>0.296721</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>7.31474</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>0.986009</v>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>24.307 (0.297x)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>7.315 (0.986x)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -650,17 +623,15 @@
       <c r="B8" s="3" t="n">
         <v>22.4732</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>110.691</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>0.203026</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>21.45362</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>1.047525</v>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>110.691 (0.203x)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>21.454 (1.048x)</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -672,17 +643,15 @@
       <c r="B9" s="3" t="n">
         <v>24.854</v>
       </c>
-      <c r="C9" s="3" t="n">
-        <v>204.421</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>0.121582</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>25.606798</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.970602</v>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>204.421 (0.122x)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>25.607 (0.971x)</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -694,17 +663,15 @@
       <c r="B10" s="3" t="n">
         <v>10.188</v>
       </c>
-      <c r="C10" s="3" t="n">
-        <v>465.801</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>0.021872</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>10.96317</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0.929293</v>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>465.801 (0.022x)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>10.963 (0.929x)</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -716,21 +683,19 @@
       <c r="B11" s="3" t="n">
         <v>8.48746</v>
       </c>
-      <c r="C11" s="3" t="n">
-        <v>1413.92</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>0.006003</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>15.82919</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.5361900000000001</v>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1,413.920 (0.006x)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>15.829 (0.536x)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -744,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -826,34 +791,46 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Speedup definition</t>
+          <t>Cell format</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GPG runtime / method runtime</t>
+          <t>Runtime in milliseconds (speedup over GPG)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Interpretation</t>
+          <t>Speedup definition</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Above 1x is faster than GPG; below 1x is slower</t>
+          <t>GPG runtime / method runtime</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Above 1x is faster than GPG; below 1x is slower</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>doc/adaptive-checkpoint-20260831-full-suite.csv</t>
         </is>

</xml_diff>